<commit_message>
Actualiza portafolio 2026-06-14 01:18 UTC
</commit_message>
<xml_diff>
--- a/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
+++ b/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="294">
   <si>
     <t xml:space="preserve">50001485-CALABRESSE METRO STO DOMINGO  </t>
   </si>
@@ -893,9 +893,6 @@
   </si>
   <si>
     <t>Pruebas instalacion componentes</t>
-  </si>
-  <si>
-    <t>Media</t>
   </si>
 </sst>
 </file>
@@ -6300,7 +6297,7 @@
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46185.16808386574</v>
+        <v>46186.20086041666</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>293</v>
@@ -6347,8 +6344,8 @@
       <c r="S82" s="6">
         <v>0</v>
       </c>
-      <c r="T82" s="12" t="s">
-        <v>294</v>
+      <c r="T82" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="U82" s="10" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-22 01:34 UTC
</commit_message>
<xml_diff>
--- a/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
+++ b/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
@@ -2881,9 +2881,11 @@
       <c r="B26" s="5">
         <v>46073.68416899306</v>
       </c>
-      <c r="C26" s="6"/>
+      <c r="C26" s="5">
+        <v>46195.06028828704</v>
+      </c>
       <c r="D26" s="5">
-        <v>46182.68409435185</v>
+        <v>46195.0603066551</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>105</v>
@@ -2917,10 +2919,12 @@
       </c>
       <c r="Q26" s="6"/>
       <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
+      <c r="S26" s="6">
+        <v>1</v>
+      </c>
       <c r="T26" s="6"/>
-      <c r="U26" s="12" t="s">
-        <v>85</v>
+      <c r="U26" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-22 21:02 UTC
</commit_message>
<xml_diff>
--- a/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
+++ b/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1019" uniqueCount="294">
   <si>
     <t xml:space="preserve">50001485-CALABRESSE METRO STO DOMINGO  </t>
   </si>
@@ -5229,9 +5229,11 @@
       <c r="B64" s="5">
         <v>46073.68417018518</v>
       </c>
-      <c r="C64" s="6"/>
+      <c r="C64" s="5">
+        <v>46195.86446399306</v>
+      </c>
       <c r="D64" s="5">
-        <v>46193.61091024306</v>
+        <v>46195.864478414354</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>235</v>
@@ -5265,9 +5267,13 @@
       </c>
       <c r="Q64" s="6"/>
       <c r="R64" s="6"/>
-      <c r="S64" s="6"/>
+      <c r="S64" s="6">
+        <v>1</v>
+      </c>
       <c r="T64" s="6"/>
-      <c r="U64" s="6"/>
+      <c r="U64" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
@@ -5471,9 +5477,11 @@
       <c r="B68" s="5">
         <v>46076.63671706019</v>
       </c>
-      <c r="C68" s="6"/>
+      <c r="C68" s="5">
+        <v>46195.86400119213</v>
+      </c>
       <c r="D68" s="5">
-        <v>46193.610651423616</v>
+        <v>46195.86401943287</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>248</v>
@@ -5518,13 +5526,13 @@
         <v>46134</v>
       </c>
       <c r="S68" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T68" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U68" s="12" t="s">
-        <v>85</v>
+      <c r="U68" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5603,7 +5611,7 @@
         <v>46193.61090479167</v>
       </c>
       <c r="D70" s="5">
-        <v>46193.61092013889</v>
+        <v>46195.864020023146</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>187</v>
@@ -5653,8 +5661,8 @@
       <c r="T70" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U70" s="11" t="s">
-        <v>33</v>
+      <c r="U70" s="12" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
@@ -5664,9 +5672,11 @@
       <c r="B71" s="8">
         <v>46073.6841718287</v>
       </c>
-      <c r="C71" s="9"/>
+      <c r="C71" s="8">
+        <v>46195.86444770833</v>
+      </c>
       <c r="D71" s="8">
-        <v>46161.17018530093</v>
+        <v>46195.86446715277</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>188</v>
@@ -5711,13 +5721,13 @@
         <v>46160</v>
       </c>
       <c r="S71" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T71" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U71" s="10" t="s">
-        <v>57</v>
+      <c r="U71" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -5776,7 +5786,7 @@
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46162.1970055787</v>
+        <v>46195.86446728009</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>262</v>
@@ -5824,8 +5834,8 @@
       <c r="T73" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U73" s="10" t="s">
-        <v>57</v>
+      <c r="U73" s="12" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-25 20:32 UTC
</commit_message>
<xml_diff>
--- a/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
+++ b/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
@@ -4869,7 +4869,7 @@
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46157.491688159724</v>
+        <v>46198.81949164352</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>190</v>
@@ -4914,9 +4914,11 @@
       <c r="B59" s="8">
         <v>46073.68416956019</v>
       </c>
-      <c r="C59" s="9"/>
+      <c r="C59" s="8">
+        <v>46198.81948427083</v>
+      </c>
       <c r="D59" s="8">
-        <v>46174.63955796296</v>
+        <v>46198.819671226855</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>221</v>
@@ -4961,13 +4963,13 @@
         <v>46125</v>
       </c>
       <c r="S59" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T59" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U59" s="12" t="s">
-        <v>85</v>
+      <c r="U59" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -5422,7 +5424,7 @@
         <v>46193.61080444444</v>
       </c>
       <c r="D67" s="8">
-        <v>46193.61083505787</v>
+        <v>46198.81950197917</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>244</v>
@@ -5472,8 +5474,8 @@
       <c r="T67" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U67" s="11" t="s">
-        <v>33</v>
+      <c r="U67" s="12" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-26 14:31 UTC
</commit_message>
<xml_diff>
--- a/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
+++ b/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1019" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1019" uniqueCount="296">
   <si>
     <t xml:space="preserve">50001485-CALABRESSE METRO STO DOMINGO  </t>
   </si>
@@ -800,6 +800,12 @@
   </si>
   <si>
     <t>Coordinacion Entrega con Cliente</t>
+  </si>
+  <si>
+    <t>Karin Pinto</t>
+  </si>
+  <si>
+    <t>kpinto@zitron.com</t>
   </si>
   <si>
     <t>Embalaje,Logistica:</t>
@@ -5794,7 +5800,7 @@
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46195.86446728009</v>
+        <v>46199.554064814816</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>262</v>
@@ -5803,10 +5809,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>36</v>
+        <v>263</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>37</v>
+        <v>264</v>
       </c>
       <c r="I73" s="9"/>
       <c r="J73" s="8">
@@ -5828,7 +5834,7 @@
         <v>188</v>
       </c>
       <c r="P73" s="9" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="Q73" s="8">
         <v>46161</v>
@@ -5848,7 +5854,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B74" s="5">
         <v>46073.68416979167</v>
@@ -5860,7 +5866,7 @@
         <v>46193.611063425924</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
@@ -5888,10 +5894,10 @@
         <v>259</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="Q74" s="5">
         <v>46162</v>
@@ -5911,7 +5917,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B75" s="8">
         <v>46073.68417006945</v>
@@ -5921,16 +5927,16 @@
         <v>46193.61106297454</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="I75" s="8">
         <v>46164</v>
@@ -5951,10 +5957,10 @@
         <v>259</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="Q75" s="8">
         <v>46164</v>
@@ -5974,7 +5980,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B76" s="5">
         <v>46073.684170347224</v>
@@ -5984,16 +5990,16 @@
         <v>46168.20800158565</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="I76" s="6"/>
       <c r="J76" s="5">
@@ -6012,10 +6018,10 @@
         <v>259</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="Q76" s="5">
         <v>46167</v>
@@ -6035,7 +6041,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B77" s="8">
         <v>46073.68417061343</v>
@@ -6045,7 +6051,7 @@
         <v>46091.7946121875</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>25</v>
@@ -6069,7 +6075,7 @@
         <v>26</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="P77" s="9" t="s">
         <v>26</v>
@@ -6082,7 +6088,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B78" s="5">
         <v>46073.68417087963</v>
@@ -6092,16 +6098,16 @@
         <v>46177.189791805555</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I78" s="5">
         <v>46168</v>
@@ -6119,13 +6125,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="Q78" s="5">
         <v>46168</v>
@@ -6145,7 +6151,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B79" s="8">
         <v>46073.68417115741</v>
@@ -6155,16 +6161,16 @@
         <v>46177.18979210648</v>
       </c>
       <c r="E79" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="F79" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G79" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="H79" s="9" t="s">
         <v>284</v>
-      </c>
-      <c r="F79" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G79" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="H79" s="9" t="s">
-        <v>282</v>
       </c>
       <c r="I79" s="8">
         <v>46168</v>
@@ -6182,13 +6188,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="Q79" s="8">
         <v>46168</v>
@@ -6208,7 +6214,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B80" s="5">
         <v>46091.74474364583</v>
@@ -6218,7 +6224,7 @@
         <v>46091.79747990741</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>25</v>
@@ -6242,7 +6248,7 @@
         <v>26</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>26</v>
@@ -6261,7 +6267,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B81" s="8">
         <v>46091.74497048611</v>
@@ -6271,7 +6277,7 @@
         <v>46177.189791620374</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
@@ -6298,13 +6304,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="Q81" s="8">
         <v>46168</v>
@@ -6324,7 +6330,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B82" s="5">
         <v>46091.7450819213</v>
@@ -6334,7 +6340,7 @@
         <v>46186.20086041666</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
@@ -6361,13 +6367,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="Q82" s="5">
         <v>46177</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-30 22:01 UTC
</commit_message>
<xml_diff>
--- a/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
+++ b/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
@@ -5753,7 +5753,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46193.611056388894</v>
+        <v>46203.90143832176</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>259</v>
@@ -5798,9 +5798,11 @@
       <c r="B73" s="8">
         <v>46073.68416949074</v>
       </c>
-      <c r="C73" s="9"/>
+      <c r="C73" s="8">
+        <v>46203.90143077546</v>
+      </c>
       <c r="D73" s="8">
-        <v>46203.56918020833</v>
+        <v>46203.90144782407</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>262</v>
@@ -5843,13 +5845,13 @@
         <v>46161</v>
       </c>
       <c r="S73" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T73" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U73" s="12" t="s">
-        <v>85</v>
+      <c r="U73" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5863,7 +5865,7 @@
         <v>46193.61104665509</v>
       </c>
       <c r="D74" s="5">
-        <v>46193.611063425924</v>
+        <v>46203.90143780093</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>267</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-06 14:11 UTC
</commit_message>
<xml_diff>
--- a/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
+++ b/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1019" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1019" uniqueCount="298">
   <si>
     <t xml:space="preserve">50001485-CALABRESSE METRO STO DOMINGO  </t>
   </si>
@@ -176,6 +176,12 @@
   </si>
   <si>
     <t>Revisión tableros pruebas</t>
+  </si>
+  <si>
+    <t>sergio saavedra fernandez</t>
+  </si>
+  <si>
+    <t>sergio.saavedra@zitron.com</t>
   </si>
   <si>
     <t>Recepcion Tableros</t>
@@ -2015,7 +2021,7 @@
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46109.14656262731</v>
+        <v>46209.58085539352</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2024,10 +2030,10 @@
         <v>26</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="I12" s="5">
         <v>46104</v>
@@ -2048,10 +2054,10 @@
         <v>46</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="Q12" s="5">
         <v>46104</v>
@@ -2066,12 +2072,12 @@
         <v>32</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B13" s="8">
         <v>46073.68417070602</v>
@@ -2083,7 +2089,7 @@
         <v>46107.80691021991</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>25</v>
@@ -2107,7 +2113,7 @@
         <v>26</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>26</v>
@@ -2124,7 +2130,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B14" s="5">
         <v>46073.684169224536</v>
@@ -2136,16 +2142,16 @@
         <v>46094.53642131944</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I14" s="5">
         <v>45987</v>
@@ -2163,13 +2169,13 @@
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>41</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="Q14" s="5">
         <v>45987</v>
@@ -2189,7 +2195,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B15" s="8">
         <v>46073.684169872686</v>
@@ -2201,16 +2207,16 @@
         <v>46100.76314293982</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I15" s="8">
         <v>45987</v>
@@ -2228,13 +2234,13 @@
         <v>26</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>41</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Q15" s="8">
         <v>45987</v>
@@ -2254,7 +2260,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B16" s="5">
         <v>46073.68417017361</v>
@@ -2266,16 +2272,16 @@
         <v>46101.81844299768</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I16" s="5">
         <v>45987</v>
@@ -2293,13 +2299,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>41</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q16" s="5">
         <v>45987</v>
@@ -2319,7 +2325,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B17" s="8">
         <v>46073.68417078703</v>
@@ -2331,16 +2337,16 @@
         <v>46107.806898807874</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I17" s="8">
         <v>45987</v>
@@ -2358,13 +2364,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="Q17" s="8">
         <v>45987</v>
@@ -2384,7 +2390,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B18" s="5">
         <v>46073.6841712037</v>
@@ -2396,7 +2402,7 @@
         <v>46107.80883890046</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>25</v>
@@ -2420,7 +2426,7 @@
         <v>26</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P18" s="6" t="s">
         <v>26</v>
@@ -2437,7 +2443,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B19" s="8">
         <v>46073.68417184028</v>
@@ -2449,16 +2455,16 @@
         <v>46094.53691905092</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I19" s="8">
         <v>45989</v>
@@ -2476,13 +2482,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Q19" s="8">
         <v>45989</v>
@@ -2502,7 +2508,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B20" s="5">
         <v>46073.68417155092</v>
@@ -2514,16 +2520,16 @@
         <v>46100.763124074074</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I20" s="5">
         <v>45999</v>
@@ -2541,13 +2547,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="Q20" s="5">
         <v>45999</v>
@@ -2562,12 +2568,12 @@
         <v>32</v>
       </c>
       <c r="U20" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B21" s="8">
         <v>46073.68417212963</v>
@@ -2579,16 +2585,16 @@
         <v>46107.80882605324</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I21" s="8">
         <v>45989</v>
@@ -2606,13 +2612,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O21" s="9" t="s">
         <v>49</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Q21" s="8">
         <v>45989</v>
@@ -2632,7 +2638,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B22" s="5">
         <v>46073.684172442125</v>
@@ -2644,16 +2650,16 @@
         <v>46100.76394396991</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I22" s="5">
         <v>45999</v>
@@ -2671,13 +2677,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="Q22" s="5">
         <v>45999</v>
@@ -2697,7 +2703,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B23" s="8">
         <v>46076.61209707176</v>
@@ -2709,16 +2715,16 @@
         <v>46107.808263576386</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I23" s="8">
         <v>45999</v>
@@ -2736,13 +2742,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="Q23" s="8">
         <v>45999</v>
@@ -2762,7 +2768,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B24" s="5">
         <v>46094.53930710648</v>
@@ -2774,7 +2780,7 @@
         <v>46106.60917302083</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>25</v>
@@ -2798,7 +2804,7 @@
         <v>26</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="P24" s="6" t="s">
         <v>26</v>
@@ -2809,7 +2815,7 @@
         <v>1</v>
       </c>
       <c r="T24" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U24" s="11" t="s">
         <v>33</v>
@@ -2817,7 +2823,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B25" s="8">
         <v>46073.68416866898</v>
@@ -2829,16 +2835,16 @@
         <v>46106.60915524306</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I25" s="8">
         <v>45999</v>
@@ -2856,13 +2862,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="Q25" s="8">
         <v>45999</v>
@@ -2874,7 +2880,7 @@
         <v>1</v>
       </c>
       <c r="T25" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U25" s="11" t="s">
         <v>33</v>
@@ -2882,7 +2888,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B26" s="5">
         <v>46073.68416899306</v>
@@ -2894,7 +2900,7 @@
         <v>46195.0603066551</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>25</v>
@@ -2918,7 +2924,7 @@
         <v>26</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>26</v>
@@ -2935,7 +2941,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B27" s="8">
         <v>46073.68416959491</v>
@@ -2947,16 +2953,16 @@
         <v>46174.62770914352</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I27" s="8">
         <v>45993</v>
@@ -2974,13 +2980,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Q27" s="8">
         <v>45993</v>
@@ -2995,12 +3001,12 @@
         <v>32</v>
       </c>
       <c r="U27" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B28" s="5">
         <v>46073.68416988426</v>
@@ -3012,16 +3018,16 @@
         <v>46107.80715059028</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I28" s="5">
         <v>45993</v>
@@ -3039,13 +3045,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
@@ -3053,15 +3059,15 @@
         <v>0</v>
       </c>
       <c r="T28" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U28" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B29" s="8">
         <v>46073.68417013889</v>
@@ -3073,16 +3079,16 @@
         <v>46174.62770383102</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I29" s="8">
         <v>46020</v>
@@ -3100,13 +3106,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="Q29" s="9"/>
       <c r="R29" s="9"/>
@@ -3114,15 +3120,15 @@
         <v>0</v>
       </c>
       <c r="T29" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U29" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B30" s="5">
         <v>46073.684170416665</v>
@@ -3134,16 +3140,16 @@
         <v>46121.89140954861</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I30" s="5">
         <v>46020</v>
@@ -3161,13 +3167,13 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
@@ -3175,15 +3181,15 @@
         <v>0</v>
       </c>
       <c r="T30" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U30" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B31" s="8">
         <v>46073.68416929398</v>
@@ -3195,16 +3201,16 @@
         <v>46174.639652604164</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I31" s="8">
         <v>46001</v>
@@ -3222,13 +3228,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Q31" s="8">
         <v>46001</v>
@@ -3248,7 +3254,7 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B32" s="5">
         <v>46073.68416954861</v>
@@ -3260,16 +3266,16 @@
         <v>46174.639389062504</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I32" s="5">
         <v>46001</v>
@@ -3287,13 +3293,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
@@ -3301,15 +3307,15 @@
         <v>0</v>
       </c>
       <c r="T32" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U32" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B33" s="8">
         <v>46073.68416979167</v>
@@ -3321,16 +3327,16 @@
         <v>46174.63953965278</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I33" s="8">
         <v>46003</v>
@@ -3348,13 +3354,13 @@
         <v>26</v>
       </c>
       <c r="N33" s="9" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P33" s="9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="Q33" s="9"/>
       <c r="R33" s="9"/>
@@ -3362,15 +3368,15 @@
         <v>0</v>
       </c>
       <c r="T33" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U33" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B34" s="5">
         <v>46073.68417075231</v>
@@ -3382,16 +3388,16 @@
         <v>46156.658810520836</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I34" s="5">
         <v>46001</v>
@@ -3409,13 +3415,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Q34" s="5">
         <v>46001</v>
@@ -3435,7 +3441,7 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B35" s="8">
         <v>46073.684171030094</v>
@@ -3447,16 +3453,16 @@
         <v>46107.80771298611</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I35" s="8">
         <v>46001</v>
@@ -3474,13 +3480,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="Q35" s="9"/>
       <c r="R35" s="9"/>
@@ -3488,15 +3494,15 @@
         <v>0</v>
       </c>
       <c r="T35" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U35" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B36" s="5">
         <v>46073.68416916666</v>
@@ -3508,16 +3514,16 @@
         <v>46156.65878615741</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I36" s="5">
         <v>46003</v>
@@ -3535,13 +3541,13 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
@@ -3549,15 +3555,15 @@
         <v>0</v>
       </c>
       <c r="T36" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U36" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B37" s="8">
         <v>46073.68417003472</v>
@@ -3569,16 +3575,16 @@
         <v>46182.68408826389</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I37" s="8">
         <v>45993</v>
@@ -3596,13 +3602,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="O37" s="9" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Q37" s="8">
         <v>46024</v>
@@ -3622,7 +3628,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B38" s="5">
         <v>46073.684170277775</v>
@@ -3634,16 +3640,16 @@
         <v>46169.8387588426</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I38" s="5">
         <v>45993</v>
@@ -3661,13 +3667,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3675,15 +3681,15 @@
         <v>0</v>
       </c>
       <c r="T38" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U38" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B39" s="8">
         <v>46073.684170520835</v>
@@ -3695,16 +3701,16 @@
         <v>46182.6840615625</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I39" s="8">
         <v>46002</v>
@@ -3722,13 +3728,13 @@
         <v>26</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="P39" s="9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Q39" s="9"/>
       <c r="R39" s="9"/>
@@ -3736,15 +3742,15 @@
         <v>0</v>
       </c>
       <c r="T39" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U39" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B40" s="5">
         <v>46076.61481881945</v>
@@ -3756,16 +3762,16 @@
         <v>46127.16789894676</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I40" s="5">
         <v>46001</v>
@@ -3783,13 +3789,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Q40" s="5">
         <v>46001</v>
@@ -3809,7 +3815,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B41" s="8">
         <v>46076.614840277776</v>
@@ -3821,16 +3827,16 @@
         <v>46107.80900657407</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I41" s="8">
         <v>46001</v>
@@ -3848,13 +3854,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="Q41" s="8">
         <v>46001</v>
@@ -3866,15 +3872,15 @@
         <v>0</v>
       </c>
       <c r="T41" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U41" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B42" s="5">
         <v>46076.6150438426</v>
@@ -3886,16 +3892,16 @@
         <v>46107.80904144676</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I42" s="5">
         <v>46044</v>
@@ -3913,13 +3919,13 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="Q42" s="5">
         <v>46044</v>
@@ -3931,15 +3937,15 @@
         <v>0</v>
       </c>
       <c r="T42" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U42" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B43" s="8">
         <v>46073.68417068287</v>
@@ -3951,16 +3957,16 @@
         <v>46154.86694947917</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H43" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I43" s="8">
         <v>46001</v>
@@ -3978,13 +3984,13 @@
         <v>26</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="P43" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Q43" s="8">
         <v>46001</v>
@@ -4004,7 +4010,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B44" s="5">
         <v>46073.6841709375</v>
@@ -4016,16 +4022,16 @@
         <v>46107.81013429398</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I44" s="5">
         <v>46001</v>
@@ -4043,13 +4049,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4057,15 +4063,15 @@
         <v>0</v>
       </c>
       <c r="T44" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U44" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B45" s="8">
         <v>46073.68417122685</v>
@@ -4077,16 +4083,16 @@
         <v>46154.866921967594</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H45" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I45" s="8">
         <v>46027</v>
@@ -4104,13 +4110,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="P45" s="9" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="Q45" s="9"/>
       <c r="R45" s="9"/>
@@ -4118,15 +4124,15 @@
         <v>0</v>
       </c>
       <c r="T45" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U45" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B46" s="5">
         <v>46073.68417148148</v>
@@ -4138,7 +4144,7 @@
         <v>46198.57100354167</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>25</v>
@@ -4162,7 +4168,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4179,7 +4185,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B47" s="8">
         <v>46073.68417173611</v>
@@ -4191,16 +4197,16 @@
         <v>46107.72069699074</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="H47" s="9" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I47" s="8">
         <v>45999</v>
@@ -4218,13 +4224,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="P47" s="9" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="Q47" s="8">
         <v>45999</v>
@@ -4244,7 +4250,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B48" s="5">
         <v>46073.68416831018</v>
@@ -4256,16 +4262,16 @@
         <v>46121.89142756944</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I48" s="5">
         <v>46063</v>
@@ -4283,13 +4289,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="Q48" s="5">
         <v>46063</v>
@@ -4304,12 +4310,12 @@
         <v>32</v>
       </c>
       <c r="U48" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B49" s="8">
         <v>46091.74401927083</v>
@@ -4321,16 +4327,16 @@
         <v>46107.72081601852</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="H49" s="9" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I49" s="9"/>
       <c r="J49" s="8">
@@ -4346,13 +4352,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="9" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="O49" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="P49" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="Q49" s="8">
         <v>46070</v>
@@ -4372,7 +4378,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B50" s="5">
         <v>46091.744054490744</v>
@@ -4384,16 +4390,16 @@
         <v>46198.57098844908</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="I50" s="5">
         <v>46157</v>
@@ -4411,13 +4417,13 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="P50" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="Q50" s="5">
         <v>46157</v>
@@ -4437,7 +4443,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B51" s="8">
         <v>46073.68416862268</v>
@@ -4449,7 +4455,7 @@
         <v>46127.77592181713</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>25</v>
@@ -4473,7 +4479,7 @@
         <v>26</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="P51" s="9" t="s">
         <v>26</v>
@@ -4490,7 +4496,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B52" s="5">
         <v>46073.68416885417</v>
@@ -4502,16 +4508,16 @@
         <v>46154.866942974535</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I52" s="5">
         <v>46057</v>
@@ -4529,13 +4535,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="Q52" s="5">
         <v>46057</v>
@@ -4550,12 +4556,12 @@
         <v>32</v>
       </c>
       <c r="U52" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B53" s="8">
         <v>46073.6841691088</v>
@@ -4567,16 +4573,16 @@
         <v>46127.77590576389</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H53" s="9" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="I53" s="8">
         <v>46062</v>
@@ -4594,13 +4600,13 @@
         <v>26</v>
       </c>
       <c r="N53" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="P53" s="9" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="Q53" s="8">
         <v>46062</v>
@@ -4620,7 +4626,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B54" s="5">
         <v>46073.68416935185</v>
@@ -4632,7 +4638,7 @@
         <v>46160.687379560186</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>25</v>
@@ -4656,7 +4662,7 @@
         <v>26</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>26</v>
@@ -4673,7 +4679,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B55" s="8">
         <v>46073.68416957176</v>
@@ -4685,16 +4691,16 @@
         <v>46157.49039020833</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="I55" s="8">
         <v>46063</v>
@@ -4712,13 +4718,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="9" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="O55" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="P55" s="9" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="Q55" s="8">
         <v>46063</v>
@@ -4738,7 +4744,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B56" s="5">
         <v>46073.68416979167</v>
@@ -4750,16 +4756,16 @@
         <v>46157.49054525463</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="I56" s="5">
         <v>46072</v>
@@ -4777,13 +4783,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="Q56" s="5">
         <v>46072</v>
@@ -4803,7 +4809,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B57" s="8">
         <v>46073.68417001158</v>
@@ -4815,16 +4821,16 @@
         <v>46160.68736836806</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="I57" s="8">
         <v>46092</v>
@@ -4842,13 +4848,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="9" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="O57" s="9" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="P57" s="9" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="Q57" s="8">
         <v>46092</v>
@@ -4868,7 +4874,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B58" s="5">
         <v>46073.68417021991</v>
@@ -4878,7 +4884,7 @@
         <v>46198.81949164352</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>25</v>
@@ -4902,7 +4908,7 @@
         <v>26</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>26</v>
@@ -4915,7 +4921,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B59" s="8">
         <v>46073.68416956019</v>
@@ -4927,16 +4933,16 @@
         <v>46198.819671226855</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I59" s="8">
         <v>46122</v>
@@ -4954,13 +4960,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="O59" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="P59" s="9" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="Q59" s="8">
         <v>46122</v>
@@ -4980,7 +4986,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B60" s="5">
         <v>46073.68417045139</v>
@@ -4992,16 +4998,16 @@
         <v>46157.49118612269</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I60" s="5">
         <v>46058</v>
@@ -5019,13 +5025,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="Q60" s="5">
         <v>46057</v>
@@ -5045,7 +5051,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B61" s="8">
         <v>46073.68416986111</v>
@@ -5057,16 +5063,16 @@
         <v>46174.6277108912</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I61" s="8">
         <v>46150</v>
@@ -5084,13 +5090,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="P61" s="9" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="Q61" s="8">
         <v>46150</v>
@@ -5105,12 +5111,12 @@
         <v>32</v>
       </c>
       <c r="U61" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B62" s="5">
         <v>46073.68416916666</v>
@@ -5120,16 +5126,16 @@
         <v>46182.684078356484</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I62" s="5">
         <v>46100</v>
@@ -5147,13 +5153,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="Q62" s="5">
         <v>46100</v>
@@ -5168,12 +5174,12 @@
         <v>32</v>
       </c>
       <c r="U62" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B63" s="8">
         <v>46076.63637116898</v>
@@ -5185,16 +5191,16 @@
         <v>46157.4916971412</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I63" s="8">
         <v>46126</v>
@@ -5212,13 +5218,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="P63" s="9" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Q63" s="8">
         <v>46126</v>
@@ -5238,7 +5244,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B64" s="5">
         <v>46073.68417018518</v>
@@ -5250,7 +5256,7 @@
         <v>46195.864478414354</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>25</v>
@@ -5274,7 +5280,7 @@
         <v>26</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="P64" s="6" t="s">
         <v>26</v>
@@ -5291,7 +5297,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B65" s="8">
         <v>46073.684170486114</v>
@@ -5303,16 +5309,16 @@
         <v>46193.61064896991</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I65" s="8">
         <v>46094</v>
@@ -5330,13 +5336,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="O65" s="9" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="Q65" s="8">
         <v>46094</v>
@@ -5356,7 +5362,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B66" s="5">
         <v>46073.68417076389</v>
@@ -5368,16 +5374,16 @@
         <v>46193.610722048616</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I66" s="5">
         <v>46154</v>
@@ -5395,13 +5401,13 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="Q66" s="5">
         <v>46154</v>
@@ -5421,7 +5427,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B67" s="8">
         <v>46073.68417101852</v>
@@ -5433,16 +5439,16 @@
         <v>46198.81950197917</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I67" s="8">
         <v>46126</v>
@@ -5460,13 +5466,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="9" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="O67" s="9" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="P67" s="9" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="Q67" s="8">
         <v>46126</v>
@@ -5481,12 +5487,12 @@
         <v>32</v>
       </c>
       <c r="U67" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B68" s="5">
         <v>46076.63671706019</v>
@@ -5498,16 +5504,16 @@
         <v>46195.86401943287</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I68" s="5">
         <v>46133</v>
@@ -5525,13 +5531,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="Q68" s="5">
         <v>46133</v>
@@ -5551,7 +5557,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B69" s="8">
         <v>46073.68417128472</v>
@@ -5563,16 +5569,16 @@
         <v>46193.610887187504</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I69" s="8">
         <v>46129</v>
@@ -5590,13 +5596,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="9" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="O69" s="9" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="P69" s="9" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="Q69" s="8">
         <v>46129</v>
@@ -5616,7 +5622,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B70" s="5">
         <v>46073.684171574074</v>
@@ -5628,16 +5634,16 @@
         <v>46195.864020023146</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I70" s="5">
         <v>46156</v>
@@ -5655,13 +5661,13 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="Q70" s="5">
         <v>46156</v>
@@ -5676,12 +5682,12 @@
         <v>32</v>
       </c>
       <c r="U70" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B71" s="8">
         <v>46073.6841718287</v>
@@ -5693,16 +5699,16 @@
         <v>46198.57098592592</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H71" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I71" s="8">
         <v>46160</v>
@@ -5720,13 +5726,13 @@
         <v>26</v>
       </c>
       <c r="N71" s="9" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="O71" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="P71" s="9" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="Q71" s="8">
         <v>46160</v>
@@ -5741,12 +5747,12 @@
         <v>32</v>
       </c>
       <c r="U71" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B72" s="5">
         <v>46073.68416913194</v>
@@ -5756,7 +5762,7 @@
         <v>46203.90143832176</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>25</v>
@@ -5780,7 +5786,7 @@
         <v>26</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>26</v>
@@ -5793,7 +5799,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B73" s="8">
         <v>46073.68416949074</v>
@@ -5805,16 +5811,16 @@
         <v>46203.90144782407</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="I73" s="9"/>
       <c r="J73" s="8">
@@ -5830,13 +5836,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="P73" s="9" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="Q73" s="8">
         <v>46161</v>
@@ -5856,7 +5862,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B74" s="5">
         <v>46073.68416979167</v>
@@ -5868,16 +5874,16 @@
         <v>46203.90143780093</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I74" s="6"/>
       <c r="J74" s="5">
@@ -5893,13 +5899,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q74" s="5">
         <v>46162</v>
@@ -5919,7 +5925,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B75" s="8">
         <v>46073.68417006945</v>
@@ -5929,16 +5935,16 @@
         <v>46193.61106297454</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I75" s="8">
         <v>46164</v>
@@ -5956,13 +5962,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="Q75" s="8">
         <v>46164</v>
@@ -5977,12 +5983,12 @@
         <v>32</v>
       </c>
       <c r="U75" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B76" s="5">
         <v>46073.684170347224</v>
@@ -5992,16 +5998,16 @@
         <v>46168.20800158565</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I76" s="6"/>
       <c r="J76" s="5">
@@ -6017,13 +6023,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="Q76" s="5">
         <v>46167</v>
@@ -6038,12 +6044,12 @@
         <v>32</v>
       </c>
       <c r="U76" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B77" s="8">
         <v>46073.68417061343</v>
@@ -6053,7 +6059,7 @@
         <v>46091.7946121875</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>25</v>
@@ -6077,7 +6083,7 @@
         <v>26</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="P77" s="9" t="s">
         <v>26</v>
@@ -6090,7 +6096,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B78" s="5">
         <v>46073.68417087963</v>
@@ -6100,16 +6106,16 @@
         <v>46177.189791805555</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="I78" s="5">
         <v>46168</v>
@@ -6127,13 +6133,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="Q78" s="5">
         <v>46168</v>
@@ -6148,12 +6154,12 @@
         <v>32</v>
       </c>
       <c r="U78" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B79" s="8">
         <v>46073.68417115741</v>
@@ -6163,16 +6169,16 @@
         <v>46177.18979210648</v>
       </c>
       <c r="E79" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="F79" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G79" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="H79" s="9" t="s">
         <v>286</v>
-      </c>
-      <c r="F79" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G79" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="H79" s="9" t="s">
-        <v>284</v>
       </c>
       <c r="I79" s="8">
         <v>46168</v>
@@ -6190,13 +6196,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="Q79" s="8">
         <v>46168</v>
@@ -6211,12 +6217,12 @@
         <v>32</v>
       </c>
       <c r="U79" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B80" s="5">
         <v>46091.74474364583</v>
@@ -6226,7 +6232,7 @@
         <v>46091.79747990741</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>25</v>
@@ -6250,7 +6256,7 @@
         <v>26</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>26</v>
@@ -6261,15 +6267,15 @@
         <v>0</v>
       </c>
       <c r="T80" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U80" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B81" s="8">
         <v>46091.74497048611</v>
@@ -6279,7 +6285,7 @@
         <v>46177.189791620374</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
@@ -6306,13 +6312,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="Q81" s="8">
         <v>46168</v>
@@ -6327,12 +6333,12 @@
         <v>32</v>
       </c>
       <c r="U81" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B82" s="5">
         <v>46091.7450819213</v>
@@ -6342,7 +6348,7 @@
         <v>46186.20086041666</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
@@ -6369,13 +6375,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="Q82" s="5">
         <v>46177</v>
@@ -6390,7 +6396,7 @@
         <v>32</v>
       </c>
       <c r="U82" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-21 21:23 UTC
</commit_message>
<xml_diff>
--- a/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
+++ b/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
@@ -5753,7 +5753,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46203.90143832176</v>
+        <v>46224.65751521991</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>259</v>
@@ -5924,9 +5924,11 @@
       <c r="B75" s="8">
         <v>46073.68417006945</v>
       </c>
-      <c r="C75" s="9"/>
+      <c r="C75" s="8">
+        <v>46224.65750255787</v>
+      </c>
       <c r="D75" s="8">
-        <v>46193.61106297454</v>
+        <v>46224.65994290509</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>271</v>
@@ -5971,13 +5973,13 @@
         <v>46164</v>
       </c>
       <c r="S75" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T75" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U75" s="12" t="s">
-        <v>87</v>
+      <c r="U75" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -5989,7 +5991,7 @@
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46168.20800158565</v>
+        <v>46224.657524803246</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>276</v>
@@ -6037,8 +6039,8 @@
       <c r="T76" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U76" s="10" t="s">
-        <v>59</v>
+      <c r="U76" s="12" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-11 14:04 UTC
</commit_message>
<xml_diff>
--- a/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
+++ b/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="289">
   <si>
     <t xml:space="preserve">50001485-CALABRESSE METRO STO DOMINGO  </t>
   </si>
@@ -190,175 +190,175 @@
     <t>Embalaje,Ingenieria Servicios:</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
+    <t>1213379939220252</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete,Analisis de costeo</t>
+  </si>
+  <si>
+    <t>1213379939220253</t>
+  </si>
+  <si>
+    <t>Ingenieria Basica Motor</t>
+  </si>
+  <si>
+    <t>Carlos Pérez</t>
+  </si>
+  <si>
+    <t>cperez@zitron.com</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
+  </si>
+  <si>
+    <t>1213379939220255</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta nucleo rodete,propuesta alabes</t>
+  </si>
+  <si>
+    <t>1213379939220256</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta sensores,propuesta compras a codigo // aprovisionamiento,Planos Preliminares</t>
+  </si>
+  <si>
+    <t>1213379939220257</t>
+  </si>
+  <si>
+    <t>Analisis de costeo</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:,Costos</t>
+  </si>
+  <si>
+    <t>1213379939220258</t>
+  </si>
+  <si>
+    <t>Propuesta compras:</t>
+  </si>
+  <si>
+    <t>propuesta motor,propuesta alabes,propuesta tableros,propuesta nucleo rodete,propuesta sensores</t>
+  </si>
+  <si>
+    <t>1213379939220260</t>
+  </si>
+  <si>
+    <t>propuesta motor</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC motor</t>
+  </si>
+  <si>
+    <t>1213379939220259</t>
+  </si>
+  <si>
+    <t>propuesta alabes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta compras:,Generación OC Alabe OT 4183 </t>
+  </si>
+  <si>
+    <t>1213379939220261</t>
+  </si>
+  <si>
+    <t>propuesta tableros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta compras:,Generación OC Tableros OT 4184 </t>
+  </si>
+  <si>
+    <t>1213379939220262</t>
+  </si>
+  <si>
+    <t>propuesta nucleo rodete</t>
+  </si>
+  <si>
+    <t>NATALYA ESPINOZA</t>
+  </si>
+  <si>
+    <t>nespinoza@zitron.com</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Rodete</t>
+  </si>
+  <si>
+    <t>1213402049404024</t>
+  </si>
+  <si>
+    <t>propuesta sensores</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC sensores</t>
+  </si>
+  <si>
+    <t>1213653245299154</t>
+  </si>
+  <si>
+    <t>Propuesta producción</t>
+  </si>
+  <si>
+    <t>propuesta compras a codigo // aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>1213379939220263</t>
+  </si>
+  <si>
+    <t>Generación OC materiales,Propuesta producción</t>
+  </si>
+  <si>
+    <t>1213379939220264</t>
+  </si>
+  <si>
+    <t>Compras:</t>
+  </si>
+  <si>
+    <t>Motor,Alabe OT 4183 ,Rodete,Tablero OT 4184,Sensores,Materiales a codigo // compras locales aprovisionamientomiento:</t>
+  </si>
+  <si>
+    <t>1213379942217192</t>
+  </si>
+  <si>
+    <t>Motor</t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>ecarico@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC motor,Planos motor proveedor,Fabricación motor</t>
+  </si>
+  <si>
+    <t>1213379942217193</t>
+  </si>
+  <si>
+    <t>Generación OC motor</t>
+  </si>
+  <si>
+    <t>Fabricación motor,Planos motor proveedor,Motor</t>
+  </si>
+  <si>
     <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1213379939220252</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete,Analisis de costeo</t>
-  </si>
-  <si>
-    <t>1213379939220253</t>
-  </si>
-  <si>
-    <t>Ingenieria Basica Motor</t>
-  </si>
-  <si>
-    <t>Carlos Pérez</t>
-  </si>
-  <si>
-    <t>cperez@zitron.com</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
-  </si>
-  <si>
-    <t>1213379939220255</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta nucleo rodete,propuesta alabes</t>
-  </si>
-  <si>
-    <t>1213379939220256</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta sensores,propuesta compras a codigo // aprovisionamiento,Planos Preliminares</t>
-  </si>
-  <si>
-    <t>1213379939220257</t>
-  </si>
-  <si>
-    <t>Analisis de costeo</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Costos</t>
-  </si>
-  <si>
-    <t>1213379939220258</t>
-  </si>
-  <si>
-    <t>Propuesta compras:</t>
-  </si>
-  <si>
-    <t>propuesta motor,propuesta alabes,propuesta tableros,propuesta nucleo rodete,propuesta sensores</t>
-  </si>
-  <si>
-    <t>1213379939220260</t>
-  </si>
-  <si>
-    <t>propuesta motor</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC motor</t>
-  </si>
-  <si>
-    <t>1213379939220259</t>
-  </si>
-  <si>
-    <t>propuesta alabes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuesta compras:,Generación OC Alabe OT 4183 </t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1213379939220261</t>
-  </si>
-  <si>
-    <t>propuesta tableros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuesta compras:,Generación OC Tableros OT 4184 </t>
-  </si>
-  <si>
-    <t>1213379939220262</t>
-  </si>
-  <si>
-    <t>propuesta nucleo rodete</t>
-  </si>
-  <si>
-    <t>NATALYA ESPINOZA</t>
-  </si>
-  <si>
-    <t>nespinoza@zitron.com</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Rodete</t>
-  </si>
-  <si>
-    <t>1213402049404024</t>
-  </si>
-  <si>
-    <t>propuesta sensores</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC sensores</t>
-  </si>
-  <si>
-    <t>1213653245299154</t>
-  </si>
-  <si>
-    <t>Propuesta producción</t>
-  </si>
-  <si>
-    <t>propuesta compras a codigo // aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Baja</t>
-  </si>
-  <si>
-    <t>1213379939220263</t>
-  </si>
-  <si>
-    <t>Generación OC materiales,Propuesta producción</t>
-  </si>
-  <si>
-    <t>1213379939220264</t>
-  </si>
-  <si>
-    <t>Compras:</t>
-  </si>
-  <si>
-    <t>Motor,Alabe OT 4183 ,Rodete,Tablero OT 4184,Sensores,Materiales a codigo // compras locales aprovisionamientomiento:</t>
-  </si>
-  <si>
-    <t>1213379942217192</t>
-  </si>
-  <si>
-    <t>Motor</t>
-  </si>
-  <si>
-    <t>Eliana</t>
-  </si>
-  <si>
-    <t>ecarico@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC motor,Planos motor proveedor,Fabricación motor</t>
-  </si>
-  <si>
-    <t>1213379942217193</t>
-  </si>
-  <si>
-    <t>Generación OC motor</t>
-  </si>
-  <si>
-    <t>Fabricación motor,Planos motor proveedor,Motor</t>
   </si>
   <si>
     <t>1213379942217194</t>
@@ -1880,9 +1880,11 @@
       <c r="B10" s="5">
         <v>46073.68416996528</v>
       </c>
-      <c r="C10" s="6"/>
+      <c r="C10" s="5">
+        <v>46245.53854005787</v>
+      </c>
       <c r="D10" s="5">
-        <v>46097.5271775</v>
+        <v>46245.53855082176</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1916,9 +1918,13 @@
       </c>
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
+      <c r="S10" s="6">
+        <v>1</v>
+      </c>
       <c r="T10" s="6"/>
-      <c r="U10" s="6"/>
+      <c r="U10" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
@@ -1992,9 +1998,11 @@
       <c r="B12" s="5">
         <v>46073.68417046296</v>
       </c>
-      <c r="C12" s="6"/>
+      <c r="C12" s="5">
+        <v>46245.53851724537</v>
+      </c>
       <c r="D12" s="5">
-        <v>46231.51739815972</v>
+        <v>46245.56632384259</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2039,12 +2047,12 @@
         <v>46108</v>
       </c>
       <c r="S12" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U12" s="10" t="s">
+      <c r="U12" s="12" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2490,7 +2498,7 @@
         <v>46094.5369466088</v>
       </c>
       <c r="D20" s="5">
-        <v>46100.763124074074</v>
+        <v>46245.566185601856</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>85</v>
@@ -2540,13 +2548,13 @@
       <c r="T20" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U20" s="12" t="s">
-        <v>87</v>
+      <c r="U20" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B21" s="8">
         <v>46073.68417212963</v>
@@ -2558,7 +2566,7 @@
         <v>46107.80882605324</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>26</v>
@@ -2591,7 +2599,7 @@
         <v>49</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="Q21" s="8">
         <v>45989</v>
@@ -2611,7 +2619,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B22" s="5">
         <v>46073.684172442125</v>
@@ -2623,16 +2631,16 @@
         <v>46223.609680486115</v>
       </c>
       <c r="E22" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G22" s="6" t="s">
+      <c r="H22" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="I22" s="5">
         <v>45999</v>
@@ -2656,7 +2664,7 @@
         <v>69</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="Q22" s="5">
         <v>45999</v>
@@ -2676,7 +2684,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B23" s="8">
         <v>46076.61209707176</v>
@@ -2688,7 +2696,7 @@
         <v>46107.808263576386</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>26</v>
@@ -2721,7 +2729,7 @@
         <v>72</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q23" s="8">
         <v>45999</v>
@@ -2741,7 +2749,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B24" s="5">
         <v>46094.53930710648</v>
@@ -2753,7 +2761,7 @@
         <v>46223.60967895833</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>25</v>
@@ -2777,7 +2785,7 @@
         <v>26</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P24" s="6" t="s">
         <v>26</v>
@@ -2788,7 +2796,7 @@
         <v>1</v>
       </c>
       <c r="T24" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U24" s="11" t="s">
         <v>33</v>
@@ -2796,7 +2804,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B25" s="8">
         <v>46073.68416866898</v>
@@ -2808,16 +2816,16 @@
         <v>46223.82438457176</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="H25" s="9" t="s">
-        <v>94</v>
       </c>
       <c r="I25" s="8">
         <v>45999</v>
@@ -2835,13 +2843,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O25" s="9" t="s">
         <v>72</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="Q25" s="8">
         <v>45999</v>
@@ -2853,7 +2861,7 @@
         <v>1</v>
       </c>
       <c r="T25" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U25" s="11" t="s">
         <v>33</v>
@@ -2861,7 +2869,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B26" s="5">
         <v>46073.68416899306</v>
@@ -2873,7 +2881,7 @@
         <v>46221.69938460648</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>25</v>
@@ -2897,7 +2905,7 @@
         <v>26</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>26</v>
@@ -2914,7 +2922,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B27" s="8">
         <v>46073.68416959491</v>
@@ -2923,19 +2931,19 @@
         <v>46121.891422581015</v>
       </c>
       <c r="D27" s="8">
-        <v>46174.62770914352</v>
+        <v>46245.56621042824</v>
       </c>
       <c r="E27" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="F27" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G27" s="9" t="s">
+      <c r="H27" s="9" t="s">
         <v>110</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="I27" s="8">
         <v>45993</v>
@@ -2953,13 +2961,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q27" s="8">
         <v>45993</v>
@@ -2973,13 +2981,13 @@
       <c r="T27" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U27" s="12" t="s">
-        <v>87</v>
+      <c r="U27" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B28" s="5">
         <v>46073.68416988426</v>
@@ -2991,16 +2999,16 @@
         <v>46107.80715059028</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="I28" s="5">
         <v>45993</v>
@@ -3018,13 +3026,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="O28" s="6" t="s">
         <v>82</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
@@ -3032,10 +3040,10 @@
         <v>0</v>
       </c>
       <c r="T28" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U28" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3058,10 +3066,10 @@
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="H29" s="9" t="s">
         <v>110</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="I29" s="8">
         <v>46020</v>
@@ -3079,10 +3087,10 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="P29" s="9" t="s">
         <v>118</v>
@@ -3093,10 +3101,10 @@
         <v>0</v>
       </c>
       <c r="T29" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U29" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3119,10 +3127,10 @@
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="I30" s="5">
         <v>46020</v>
@@ -3140,10 +3148,10 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="P30" s="6" t="s">
         <v>121</v>
@@ -3154,10 +3162,10 @@
         <v>0</v>
       </c>
       <c r="T30" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U30" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -3180,10 +3188,10 @@
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>110</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="I31" s="8">
         <v>46001</v>
@@ -3201,13 +3209,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O31" s="9" t="s">
         <v>124</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q31" s="8">
         <v>46001</v>
@@ -3245,10 +3253,10 @@
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="I32" s="5">
         <v>46001</v>
@@ -3280,10 +3288,10 @@
         <v>0</v>
       </c>
       <c r="T32" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U32" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -3306,10 +3314,10 @@
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>110</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="I33" s="8">
         <v>46003</v>
@@ -3341,10 +3349,10 @@
         <v>0</v>
       </c>
       <c r="T33" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U33" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -3367,10 +3375,10 @@
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="I34" s="5">
         <v>46001</v>
@@ -3388,13 +3396,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>133</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q34" s="5">
         <v>46001</v>
@@ -3432,10 +3440,10 @@
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="H35" s="9" t="s">
         <v>110</v>
-      </c>
-      <c r="H35" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="I35" s="8">
         <v>46001</v>
@@ -3456,7 +3464,7 @@
         <v>132</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="P35" s="9" t="s">
         <v>136</v>
@@ -3467,10 +3475,10 @@
         <v>0</v>
       </c>
       <c r="T35" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U35" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -3493,10 +3501,10 @@
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="I36" s="5">
         <v>46003</v>
@@ -3528,10 +3536,10 @@
         <v>0</v>
       </c>
       <c r="T36" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U36" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -3554,10 +3562,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="H37" s="9" t="s">
         <v>110</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="I37" s="8">
         <v>45993</v>
@@ -3575,13 +3583,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O37" s="9" t="s">
         <v>142</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q37" s="8">
         <v>46024</v>
@@ -3619,10 +3627,10 @@
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H38" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="I38" s="5">
         <v>45993</v>
@@ -3643,7 +3651,7 @@
         <v>141</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>145</v>
@@ -3654,10 +3662,10 @@
         <v>0</v>
       </c>
       <c r="T38" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U38" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
@@ -3680,10 +3688,10 @@
         <v>26</v>
       </c>
       <c r="G39" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="H39" s="9" t="s">
         <v>110</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="I39" s="8">
         <v>46002</v>
@@ -3715,10 +3723,10 @@
         <v>0</v>
       </c>
       <c r="T39" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U39" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
@@ -3762,13 +3770,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>153</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q40" s="5">
         <v>46001</v>
@@ -3830,7 +3838,7 @@
         <v>150</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P41" s="9" t="s">
         <v>156</v>
@@ -3845,10 +3853,10 @@
         <v>0</v>
       </c>
       <c r="T41" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U41" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
@@ -3910,10 +3918,10 @@
         <v>0</v>
       </c>
       <c r="T42" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U42" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
@@ -3957,13 +3965,13 @@
         <v>26</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O43" s="9" t="s">
         <v>162</v>
       </c>
       <c r="P43" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q43" s="8">
         <v>46001</v>
@@ -4025,7 +4033,7 @@
         <v>161</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>165</v>
@@ -4036,10 +4044,10 @@
         <v>0</v>
       </c>
       <c r="T44" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U44" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
@@ -4097,10 +4105,10 @@
         <v>0</v>
       </c>
       <c r="T45" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U45" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
@@ -4232,7 +4240,7 @@
         <v>46107.720755358794</v>
       </c>
       <c r="D48" s="5">
-        <v>46121.89142756944</v>
+        <v>46245.566249745374</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>178</v>
@@ -4282,8 +4290,8 @@
       <c r="T48" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U48" s="12" t="s">
-        <v>87</v>
+      <c r="U48" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -4529,7 +4537,7 @@
         <v>32</v>
       </c>
       <c r="U52" s="12" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
@@ -4852,9 +4860,11 @@
       <c r="B58" s="5">
         <v>46073.68417021991</v>
       </c>
-      <c r="C58" s="6"/>
+      <c r="C58" s="5">
+        <v>46245.56632902777</v>
+      </c>
       <c r="D58" s="5">
-        <v>46198.81949164352</v>
+        <v>46245.56634005787</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>191</v>
@@ -4888,9 +4898,13 @@
       </c>
       <c r="Q58" s="6"/>
       <c r="R58" s="6"/>
-      <c r="S58" s="6"/>
+      <c r="S58" s="6">
+        <v>1</v>
+      </c>
       <c r="T58" s="6"/>
-      <c r="U58" s="6"/>
+      <c r="U58" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
@@ -5033,7 +5047,7 @@
         <v>46121.89161474537</v>
       </c>
       <c r="D61" s="8">
-        <v>46174.6277108912</v>
+        <v>46245.566324942134</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>228</v>
@@ -5083,8 +5097,8 @@
       <c r="T61" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U61" s="12" t="s">
-        <v>87</v>
+      <c r="U61" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5094,9 +5108,11 @@
       <c r="B62" s="5">
         <v>46073.68416916666</v>
       </c>
-      <c r="C62" s="6"/>
+      <c r="C62" s="5">
+        <v>46245.566306967594</v>
+      </c>
       <c r="D62" s="5">
-        <v>46182.684078356484</v>
+        <v>46245.56632961806</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>57</v>
@@ -5141,13 +5157,13 @@
         <v>46101</v>
       </c>
       <c r="S62" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T62" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U62" s="12" t="s">
-        <v>87</v>
+      <c r="U62" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -5288,10 +5304,10 @@
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H65" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="H65" s="9" t="s">
-        <v>94</v>
       </c>
       <c r="I65" s="8">
         <v>46094</v>
@@ -5353,10 +5369,10 @@
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H66" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="I66" s="5">
         <v>46154</v>
@@ -5418,10 +5434,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H67" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="H67" s="9" t="s">
-        <v>94</v>
       </c>
       <c r="I67" s="8">
         <v>46126</v>
@@ -5483,10 +5499,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="I68" s="5">
         <v>46133</v>
@@ -5548,10 +5564,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H69" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="H69" s="9" t="s">
-        <v>94</v>
       </c>
       <c r="I69" s="8">
         <v>46129</v>
@@ -5613,10 +5629,10 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H70" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="I70" s="5">
         <v>46156</v>
@@ -5678,10 +5694,10 @@
         <v>26</v>
       </c>
       <c r="G71" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H71" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="H71" s="9" t="s">
-        <v>94</v>
       </c>
       <c r="I71" s="8">
         <v>46160</v>
@@ -5732,7 +5748,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46224.65751521991</v>
+        <v>46245.56589759259</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>260</v>
@@ -5840,11 +5856,9 @@
       <c r="B74" s="5">
         <v>46073.68416979167</v>
       </c>
-      <c r="C74" s="5">
-        <v>46193.61104665509</v>
-      </c>
+      <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46223.61002724537</v>
+        <v>46245.56589204861</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>268</v>
@@ -5853,10 +5867,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="I74" s="6"/>
       <c r="J74" s="5">
@@ -5892,8 +5906,8 @@
       <c r="T74" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U74" s="11" t="s">
-        <v>33</v>
+      <c r="U74" s="12" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -5907,7 +5921,7 @@
         <v>46224.65750255787</v>
       </c>
       <c r="D75" s="8">
-        <v>46224.65994290509</v>
+        <v>46245.56589712963</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>272</v>
@@ -6019,7 +6033,7 @@
         <v>32</v>
       </c>
       <c r="U76" s="12" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -6129,7 +6143,7 @@
         <v>32</v>
       </c>
       <c r="U78" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6192,7 +6206,7 @@
         <v>32</v>
       </c>
       <c r="U79" s="10" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-11 21:01 UTC
</commit_message>
<xml_diff>
--- a/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
+++ b/data/50001485 - CALABRESSE METRO STO DOMINGO.xlsx
@@ -190,421 +190,421 @@
     <t>Embalaje,Ingenieria Servicios:</t>
   </si>
   <si>
+    <t>1213379939220252</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete,Analisis de costeo</t>
+  </si>
+  <si>
+    <t>1213379939220253</t>
+  </si>
+  <si>
+    <t>Ingenieria Basica Motor</t>
+  </si>
+  <si>
+    <t>Carlos Pérez</t>
+  </si>
+  <si>
+    <t>cperez@zitron.com</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
+  </si>
+  <si>
+    <t>1213379939220255</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta nucleo rodete,propuesta alabes</t>
+  </si>
+  <si>
+    <t>1213379939220256</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta sensores,propuesta compras a codigo // aprovisionamiento,Planos Preliminares</t>
+  </si>
+  <si>
+    <t>1213379939220257</t>
+  </si>
+  <si>
+    <t>Analisis de costeo</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:,Costos</t>
+  </si>
+  <si>
+    <t>1213379939220258</t>
+  </si>
+  <si>
+    <t>Propuesta compras:</t>
+  </si>
+  <si>
+    <t>propuesta motor,propuesta alabes,propuesta tableros,propuesta nucleo rodete,propuesta sensores</t>
+  </si>
+  <si>
+    <t>1213379939220260</t>
+  </si>
+  <si>
+    <t>propuesta motor</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC motor</t>
+  </si>
+  <si>
+    <t>1213379939220259</t>
+  </si>
+  <si>
+    <t>propuesta alabes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta compras:,Generación OC Alabe OT 4183 </t>
+  </si>
+  <si>
+    <t>1213379939220261</t>
+  </si>
+  <si>
+    <t>propuesta tableros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta compras:,Generación OC Tableros OT 4184 </t>
+  </si>
+  <si>
+    <t>1213379939220262</t>
+  </si>
+  <si>
+    <t>propuesta nucleo rodete</t>
+  </si>
+  <si>
+    <t>NATALYA ESPINOZA</t>
+  </si>
+  <si>
+    <t>nespinoza@zitron.com</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Rodete</t>
+  </si>
+  <si>
+    <t>1213402049404024</t>
+  </si>
+  <si>
+    <t>propuesta sensores</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC sensores</t>
+  </si>
+  <si>
+    <t>1213653245299154</t>
+  </si>
+  <si>
+    <t>Propuesta producción</t>
+  </si>
+  <si>
+    <t>propuesta compras a codigo // aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>1213379939220263</t>
+  </si>
+  <si>
+    <t>Generación OC materiales,Propuesta producción</t>
+  </si>
+  <si>
+    <t>1213379939220264</t>
+  </si>
+  <si>
+    <t>Compras:</t>
+  </si>
+  <si>
+    <t>Motor,Alabe OT 4183 ,Rodete,Tablero OT 4184,Sensores,Materiales a codigo // compras locales aprovisionamientomiento:</t>
+  </si>
+  <si>
+    <t>1213379942217192</t>
+  </si>
+  <si>
+    <t>Motor</t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>ecarico@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC motor,Planos motor proveedor,Fabricación motor</t>
+  </si>
+  <si>
+    <t>1213379942217193</t>
+  </si>
+  <si>
+    <t>Generación OC motor</t>
+  </si>
+  <si>
+    <t>Fabricación motor,Planos motor proveedor,Motor</t>
+  </si>
+  <si>
+    <t>Tarea sin iniciar</t>
+  </si>
+  <si>
+    <t>1213379942217194</t>
+  </si>
+  <si>
+    <t>Fabricación motor</t>
+  </si>
+  <si>
+    <t>Motor,Recepcion motor</t>
+  </si>
+  <si>
+    <t>1213379942217195</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor</t>
+  </si>
+  <si>
+    <t>Motor,Planos Definitivos</t>
+  </si>
+  <si>
+    <t>1213379942217183</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alabe OT 4183 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC Alabe OT 4183 ,Fabricación Alabe OT 4183 </t>
+  </si>
+  <si>
+    <t>1213379942217184</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC Alabe OT 4183 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Alabe OT 4183 ,Alabe OT 4183 </t>
+  </si>
+  <si>
+    <t>1213379942217185</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Alabe OT 4183 </t>
+  </si>
+  <si>
+    <t>Alabe OT 4183 ,Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>1213379942217189</t>
+  </si>
+  <si>
+    <t>Rodete</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete,Fabricación Rodete</t>
+  </si>
+  <si>
+    <t>1213379942217190</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete,Rodete</t>
+  </si>
+  <si>
+    <t>1213379942217191</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete</t>
+  </si>
+  <si>
+    <t>Rodete,Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>1213379942217186</t>
+  </si>
+  <si>
+    <t>Tablero OT 4184</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC Tableros OT 4184 ,Fabricación Tablero OT 4184 </t>
+  </si>
+  <si>
+    <t>1213379942217187</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC Tableros OT 4184 </t>
+  </si>
+  <si>
+    <t>Fabricación Tablero OT 4184 ,Tablero OT 4184</t>
+  </si>
+  <si>
+    <t>1213379942217188</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Tablero OT 4184 </t>
+  </si>
+  <si>
+    <t>Tablero OT 4184,Recepcion Tableros</t>
+  </si>
+  <si>
+    <t>1213402049404030</t>
+  </si>
+  <si>
+    <t>Sensores</t>
+  </si>
+  <si>
+    <t>Yerlia Ayleen Castillo Diaz</t>
+  </si>
+  <si>
+    <t>yerlia.castillo@zitron.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC sensores,Fabricación sensores </t>
+  </si>
+  <si>
+    <t>1213402049404031</t>
+  </si>
+  <si>
+    <t>Generación OC sensores</t>
+  </si>
+  <si>
+    <t>Fabricación sensores ,Sensores</t>
+  </si>
+  <si>
+    <t>1213402049404032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación sensores </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensores,Recepción Sensores </t>
+  </si>
+  <si>
+    <t>1213379942217196</t>
+  </si>
+  <si>
+    <t>Materiales a codigo // compras locales aprovisionamientomiento:</t>
+  </si>
+  <si>
+    <t>Generación OC materiales,Fabricacion a codigo y compras locales</t>
+  </si>
+  <si>
+    <t>1213379942217197</t>
+  </si>
+  <si>
+    <t>Generación OC materiales</t>
+  </si>
+  <si>
+    <t>Fabricacion a codigo y compras locales,Materiales a codigo // compras locales aprovisionamientomiento:</t>
+  </si>
+  <si>
+    <t>1213379942217198</t>
+  </si>
+  <si>
+    <t>Fabricacion a codigo y compras locales</t>
+  </si>
+  <si>
+    <t>Materiales a codigo // compras locales aprovisionamientomiento:,Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>1213379942217199</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseño:</t>
+  </si>
+  <si>
+    <t>Planos Preliminares,Planos Definitivos</t>
+  </si>
+  <si>
+    <t>1213379942217200</t>
+  </si>
+  <si>
+    <t>Planos Preliminares</t>
+  </si>
+  <si>
+    <t>Hernan Roberto Gutierrez Barrientos</t>
+  </si>
+  <si>
+    <t>hgutierrez@zitron.com</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseño:,Planos Definitivos</t>
+  </si>
+  <si>
+    <t>1213379942217201</t>
+  </si>
+  <si>
+    <t>Planos Definitivos</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor,Planos Preliminares</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseño:,Check Planos</t>
+  </si>
+  <si>
+    <t>1213595645393569</t>
+  </si>
+  <si>
+    <t>Check Planos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control de calidad Armado,Armado,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensores </t>
+  </si>
+  <si>
+    <t>1213595645393570</t>
+  </si>
+  <si>
+    <t>Check Pruebas Fat</t>
+  </si>
+  <si>
+    <t>Francisca González Cornejo</t>
+  </si>
+  <si>
+    <t>francisca.gonzalez@zitron.com</t>
+  </si>
+  <si>
+    <t>Pruebas FAT</t>
+  </si>
+  <si>
+    <t>RE-PINTADO</t>
+  </si>
+  <si>
+    <t>1213379942217202</t>
+  </si>
+  <si>
+    <t>Bodega:</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento,Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
+  </si>
+  <si>
+    <t>1213379942217203</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Victor Muñoz</t>
+  </si>
+  <si>
+    <t>victor.munoz@zitron.com</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Bodega:</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1213379939220252</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete,Analisis de costeo</t>
-  </si>
-  <si>
-    <t>1213379939220253</t>
-  </si>
-  <si>
-    <t>Ingenieria Basica Motor</t>
-  </si>
-  <si>
-    <t>Carlos Pérez</t>
-  </si>
-  <si>
-    <t>cperez@zitron.com</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
-  </si>
-  <si>
-    <t>1213379939220255</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta nucleo rodete,propuesta alabes</t>
-  </si>
-  <si>
-    <t>1213379939220256</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta sensores,propuesta compras a codigo // aprovisionamiento,Planos Preliminares</t>
-  </si>
-  <si>
-    <t>1213379939220257</t>
-  </si>
-  <si>
-    <t>Analisis de costeo</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Costos</t>
-  </si>
-  <si>
-    <t>1213379939220258</t>
-  </si>
-  <si>
-    <t>Propuesta compras:</t>
-  </si>
-  <si>
-    <t>propuesta motor,propuesta alabes,propuesta tableros,propuesta nucleo rodete,propuesta sensores</t>
-  </si>
-  <si>
-    <t>1213379939220260</t>
-  </si>
-  <si>
-    <t>propuesta motor</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC motor</t>
-  </si>
-  <si>
-    <t>1213379939220259</t>
-  </si>
-  <si>
-    <t>propuesta alabes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuesta compras:,Generación OC Alabe OT 4183 </t>
-  </si>
-  <si>
-    <t>1213379939220261</t>
-  </si>
-  <si>
-    <t>propuesta tableros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuesta compras:,Generación OC Tableros OT 4184 </t>
-  </si>
-  <si>
-    <t>1213379939220262</t>
-  </si>
-  <si>
-    <t>propuesta nucleo rodete</t>
-  </si>
-  <si>
-    <t>NATALYA ESPINOZA</t>
-  </si>
-  <si>
-    <t>nespinoza@zitron.com</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Rodete</t>
-  </si>
-  <si>
-    <t>1213402049404024</t>
-  </si>
-  <si>
-    <t>propuesta sensores</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC sensores</t>
-  </si>
-  <si>
-    <t>1213653245299154</t>
-  </si>
-  <si>
-    <t>Propuesta producción</t>
-  </si>
-  <si>
-    <t>propuesta compras a codigo // aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Baja</t>
-  </si>
-  <si>
-    <t>1213379939220263</t>
-  </si>
-  <si>
-    <t>Generación OC materiales,Propuesta producción</t>
-  </si>
-  <si>
-    <t>1213379939220264</t>
-  </si>
-  <si>
-    <t>Compras:</t>
-  </si>
-  <si>
-    <t>Motor,Alabe OT 4183 ,Rodete,Tablero OT 4184,Sensores,Materiales a codigo // compras locales aprovisionamientomiento:</t>
-  </si>
-  <si>
-    <t>1213379942217192</t>
-  </si>
-  <si>
-    <t>Motor</t>
-  </si>
-  <si>
-    <t>Eliana</t>
-  </si>
-  <si>
-    <t>ecarico@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC motor,Planos motor proveedor,Fabricación motor</t>
-  </si>
-  <si>
-    <t>1213379942217193</t>
-  </si>
-  <si>
-    <t>Generación OC motor</t>
-  </si>
-  <si>
-    <t>Fabricación motor,Planos motor proveedor,Motor</t>
-  </si>
-  <si>
-    <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1213379942217194</t>
-  </si>
-  <si>
-    <t>Fabricación motor</t>
-  </si>
-  <si>
-    <t>Motor,Recepcion motor</t>
-  </si>
-  <si>
-    <t>1213379942217195</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor</t>
-  </si>
-  <si>
-    <t>Motor,Planos Definitivos</t>
-  </si>
-  <si>
-    <t>1213379942217183</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alabe OT 4183 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC Alabe OT 4183 ,Fabricación Alabe OT 4183 </t>
-  </si>
-  <si>
-    <t>1213379942217184</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC Alabe OT 4183 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Alabe OT 4183 ,Alabe OT 4183 </t>
-  </si>
-  <si>
-    <t>1213379942217185</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Alabe OT 4183 </t>
-  </si>
-  <si>
-    <t>Alabe OT 4183 ,Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>1213379942217189</t>
-  </si>
-  <si>
-    <t>Rodete</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete,Fabricación Rodete</t>
-  </si>
-  <si>
-    <t>1213379942217190</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete,Rodete</t>
-  </si>
-  <si>
-    <t>1213379942217191</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete</t>
-  </si>
-  <si>
-    <t>Rodete,Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>1213379942217186</t>
-  </si>
-  <si>
-    <t>Tablero OT 4184</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC Tableros OT 4184 ,Fabricación Tablero OT 4184 </t>
-  </si>
-  <si>
-    <t>1213379942217187</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC Tableros OT 4184 </t>
-  </si>
-  <si>
-    <t>Fabricación Tablero OT 4184 ,Tablero OT 4184</t>
-  </si>
-  <si>
-    <t>1213379942217188</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Tablero OT 4184 </t>
-  </si>
-  <si>
-    <t>Tablero OT 4184,Recepcion Tableros</t>
-  </si>
-  <si>
-    <t>1213402049404030</t>
-  </si>
-  <si>
-    <t>Sensores</t>
-  </si>
-  <si>
-    <t>Yerlia Ayleen Castillo Diaz</t>
-  </si>
-  <si>
-    <t>yerlia.castillo@zitron.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC sensores,Fabricación sensores </t>
-  </si>
-  <si>
-    <t>1213402049404031</t>
-  </si>
-  <si>
-    <t>Generación OC sensores</t>
-  </si>
-  <si>
-    <t>Fabricación sensores ,Sensores</t>
-  </si>
-  <si>
-    <t>1213402049404032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación sensores </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensores,Recepción Sensores </t>
-  </si>
-  <si>
-    <t>1213379942217196</t>
-  </si>
-  <si>
-    <t>Materiales a codigo // compras locales aprovisionamientomiento:</t>
-  </si>
-  <si>
-    <t>Generación OC materiales,Fabricacion a codigo y compras locales</t>
-  </si>
-  <si>
-    <t>1213379942217197</t>
-  </si>
-  <si>
-    <t>Generación OC materiales</t>
-  </si>
-  <si>
-    <t>Fabricacion a codigo y compras locales,Materiales a codigo // compras locales aprovisionamientomiento:</t>
-  </si>
-  <si>
-    <t>1213379942217198</t>
-  </si>
-  <si>
-    <t>Fabricacion a codigo y compras locales</t>
-  </si>
-  <si>
-    <t>Materiales a codigo // compras locales aprovisionamientomiento:,Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>1213379942217199</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseño:</t>
-  </si>
-  <si>
-    <t>Planos Preliminares,Planos Definitivos</t>
-  </si>
-  <si>
-    <t>1213379942217200</t>
-  </si>
-  <si>
-    <t>Planos Preliminares</t>
-  </si>
-  <si>
-    <t>Hernan Roberto Gutierrez Barrientos</t>
-  </si>
-  <si>
-    <t>hgutierrez@zitron.com</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseño:,Planos Definitivos</t>
-  </si>
-  <si>
-    <t>1213379942217201</t>
-  </si>
-  <si>
-    <t>Planos Definitivos</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor,Planos Preliminares</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseño:,Check Planos</t>
-  </si>
-  <si>
-    <t>1213595645393569</t>
-  </si>
-  <si>
-    <t>Check Planos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Control de calidad Armado,Armado,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensores </t>
-  </si>
-  <si>
-    <t>1213595645393570</t>
-  </si>
-  <si>
-    <t>Check Pruebas Fat</t>
-  </si>
-  <si>
-    <t>Francisca González Cornejo</t>
-  </si>
-  <si>
-    <t>francisca.gonzalez@zitron.com</t>
-  </si>
-  <si>
-    <t>Pruebas FAT</t>
-  </si>
-  <si>
-    <t>RE-PINTADO</t>
-  </si>
-  <si>
-    <t>1213379942217202</t>
-  </si>
-  <si>
-    <t>Bodega:</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento,Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
-  </si>
-  <si>
-    <t>1213379942217203</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Victor Muñoz</t>
-  </si>
-  <si>
-    <t>victor.munoz@zitron.com</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Bodega:</t>
   </si>
   <si>
     <t>1213379942217204</t>
@@ -2002,7 +2002,7 @@
         <v>46245.53851724537</v>
       </c>
       <c r="D12" s="5">
-        <v>46245.56632384259</v>
+        <v>46245.75325376158</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>54</v>
@@ -2052,13 +2052,13 @@
       <c r="T12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U12" s="12" t="s">
-        <v>59</v>
+      <c r="U12" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="8">
         <v>46073.68417070602</v>
@@ -2070,7 +2070,7 @@
         <v>46107.80691021991</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>25</v>
@@ -2094,7 +2094,7 @@
         <v>26</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>26</v>
@@ -2111,7 +2111,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B14" s="5">
         <v>46073.684169224536</v>
@@ -2123,16 +2123,16 @@
         <v>46094.53642131944</v>
       </c>
       <c r="E14" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="I14" s="5">
         <v>45987</v>
@@ -2150,13 +2150,13 @@
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>41</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q14" s="5">
         <v>45987</v>
@@ -2176,7 +2176,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B15" s="8">
         <v>46073.684169872686</v>
@@ -2188,16 +2188,16 @@
         <v>46100.76314293982</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G15" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H15" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="I15" s="8">
         <v>45987</v>
@@ -2215,13 +2215,13 @@
         <v>26</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>41</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Q15" s="8">
         <v>45987</v>
@@ -2241,7 +2241,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B16" s="5">
         <v>46073.68417017361</v>
@@ -2253,16 +2253,16 @@
         <v>46101.81844299768</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G16" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="I16" s="5">
         <v>45987</v>
@@ -2280,13 +2280,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>41</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q16" s="5">
         <v>45987</v>
@@ -2306,7 +2306,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B17" s="8">
         <v>46073.68417078703</v>
@@ -2318,16 +2318,16 @@
         <v>46107.806898807874</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G17" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H17" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="I17" s="8">
         <v>45987</v>
@@ -2345,13 +2345,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O17" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="P17" s="9" t="s">
         <v>76</v>
-      </c>
-      <c r="P17" s="9" t="s">
-        <v>77</v>
       </c>
       <c r="Q17" s="8">
         <v>45987</v>
@@ -2371,7 +2371,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B18" s="5">
         <v>46073.6841712037</v>
@@ -2383,7 +2383,7 @@
         <v>46107.80883890046</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>25</v>
@@ -2407,7 +2407,7 @@
         <v>26</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P18" s="6" t="s">
         <v>26</v>
@@ -2424,7 +2424,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B19" s="8">
         <v>46073.68417184028</v>
@@ -2436,16 +2436,16 @@
         <v>46094.53691905092</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G19" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H19" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="H19" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="I19" s="8">
         <v>45989</v>
@@ -2463,13 +2463,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="Q19" s="8">
         <v>45989</v>
@@ -2489,7 +2489,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B20" s="5">
         <v>46073.68417155092</v>
@@ -2501,16 +2501,16 @@
         <v>46245.566185601856</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G20" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="I20" s="5">
         <v>45999</v>
@@ -2528,13 +2528,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="Q20" s="5">
         <v>45999</v>
@@ -2554,7 +2554,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B21" s="8">
         <v>46073.68417212963</v>
@@ -2566,16 +2566,16 @@
         <v>46107.80882605324</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G21" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H21" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="I21" s="8">
         <v>45989</v>
@@ -2593,13 +2593,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O21" s="9" t="s">
         <v>49</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="Q21" s="8">
         <v>45989</v>
@@ -2619,7 +2619,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B22" s="5">
         <v>46073.684172442125</v>
@@ -2631,16 +2631,16 @@
         <v>46223.609680486115</v>
       </c>
       <c r="E22" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G22" s="6" t="s">
+      <c r="H22" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="I22" s="5">
         <v>45999</v>
@@ -2658,13 +2658,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="Q22" s="5">
         <v>45999</v>
@@ -2684,7 +2684,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B23" s="8">
         <v>46076.61209707176</v>
@@ -2696,16 +2696,16 @@
         <v>46107.808263576386</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="I23" s="8">
         <v>45999</v>
@@ -2723,13 +2723,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Q23" s="8">
         <v>45999</v>
@@ -2749,7 +2749,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B24" s="5">
         <v>46094.53930710648</v>
@@ -2761,7 +2761,7 @@
         <v>46223.60967895833</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>25</v>
@@ -2785,7 +2785,7 @@
         <v>26</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P24" s="6" t="s">
         <v>26</v>
@@ -2796,7 +2796,7 @@
         <v>1</v>
       </c>
       <c r="T24" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U24" s="11" t="s">
         <v>33</v>
@@ -2804,7 +2804,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B25" s="8">
         <v>46073.68416866898</v>
@@ -2816,16 +2816,16 @@
         <v>46223.82438457176</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>92</v>
-      </c>
-      <c r="H25" s="9" t="s">
-        <v>93</v>
       </c>
       <c r="I25" s="8">
         <v>45999</v>
@@ -2843,13 +2843,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="Q25" s="8">
         <v>45999</v>
@@ -2861,7 +2861,7 @@
         <v>1</v>
       </c>
       <c r="T25" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U25" s="11" t="s">
         <v>33</v>
@@ -2869,7 +2869,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B26" s="5">
         <v>46073.68416899306</v>
@@ -2881,7 +2881,7 @@
         <v>46221.69938460648</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>25</v>
@@ -2905,7 +2905,7 @@
         <v>26</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>26</v>
@@ -2922,7 +2922,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B27" s="8">
         <v>46073.68416959491</v>
@@ -2934,16 +2934,16 @@
         <v>46245.56621042824</v>
       </c>
       <c r="E27" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="F27" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G27" s="9" t="s">
+      <c r="H27" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="I27" s="8">
         <v>45993</v>
@@ -2961,13 +2961,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Q27" s="8">
         <v>45993</v>
@@ -2987,7 +2987,7 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B28" s="5">
         <v>46073.68416988426</v>
@@ -2999,16 +2999,16 @@
         <v>46107.80715059028</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="I28" s="5">
         <v>45993</v>
@@ -3026,13 +3026,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
@@ -3040,15 +3040,15 @@
         <v>0</v>
       </c>
       <c r="T28" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U28" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B29" s="8">
         <v>46073.68417013889</v>
@@ -3060,16 +3060,16 @@
         <v>46174.62770383102</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="H29" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="I29" s="8">
         <v>46020</v>
@@ -3087,13 +3087,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Q29" s="9"/>
       <c r="R29" s="9"/>
@@ -3101,15 +3101,15 @@
         <v>0</v>
       </c>
       <c r="T29" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U29" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B30" s="5">
         <v>46073.684170416665</v>
@@ -3121,16 +3121,16 @@
         <v>46121.89140954861</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="I30" s="5">
         <v>46020</v>
@@ -3148,13 +3148,13 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
@@ -3162,15 +3162,15 @@
         <v>0</v>
       </c>
       <c r="T30" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U30" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B31" s="8">
         <v>46073.68416929398</v>
@@ -3182,16 +3182,16 @@
         <v>46174.639652604164</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="I31" s="8">
         <v>46001</v>
@@ -3209,13 +3209,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Q31" s="8">
         <v>46001</v>
@@ -3235,7 +3235,7 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B32" s="5">
         <v>46073.68416954861</v>
@@ -3247,16 +3247,16 @@
         <v>46174.639389062504</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="I32" s="5">
         <v>46001</v>
@@ -3274,13 +3274,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
@@ -3288,15 +3288,15 @@
         <v>0</v>
       </c>
       <c r="T32" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U32" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B33" s="8">
         <v>46073.68416979167</v>
@@ -3308,16 +3308,16 @@
         <v>46174.63953965278</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="I33" s="8">
         <v>46003</v>
@@ -3335,13 +3335,13 @@
         <v>26</v>
       </c>
       <c r="N33" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P33" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Q33" s="9"/>
       <c r="R33" s="9"/>
@@ -3349,15 +3349,15 @@
         <v>0</v>
       </c>
       <c r="T33" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U33" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B34" s="5">
         <v>46073.68417075231</v>
@@ -3369,16 +3369,16 @@
         <v>46156.658810520836</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="I34" s="5">
         <v>46001</v>
@@ -3396,13 +3396,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Q34" s="5">
         <v>46001</v>
@@ -3422,7 +3422,7 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B35" s="8">
         <v>46073.684171030094</v>
@@ -3434,16 +3434,16 @@
         <v>46107.80771298611</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="H35" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="H35" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="I35" s="8">
         <v>46001</v>
@@ -3461,13 +3461,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Q35" s="9"/>
       <c r="R35" s="9"/>
@@ -3475,15 +3475,15 @@
         <v>0</v>
       </c>
       <c r="T35" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U35" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B36" s="5">
         <v>46073.68416916666</v>
@@ -3495,16 +3495,16 @@
         <v>46156.65878615741</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="I36" s="5">
         <v>46003</v>
@@ -3522,13 +3522,13 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
@@ -3536,15 +3536,15 @@
         <v>0</v>
       </c>
       <c r="T36" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U36" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B37" s="8">
         <v>46073.68417003472</v>
@@ -3556,16 +3556,16 @@
         <v>46182.68408826389</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="H37" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="I37" s="8">
         <v>45993</v>
@@ -3583,13 +3583,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O37" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Q37" s="8">
         <v>46024</v>
@@ -3609,7 +3609,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B38" s="5">
         <v>46073.684170277775</v>
@@ -3621,16 +3621,16 @@
         <v>46169.8387588426</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H38" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="I38" s="5">
         <v>45993</v>
@@ -3648,13 +3648,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3662,15 +3662,15 @@
         <v>0</v>
       </c>
       <c r="T38" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U38" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B39" s="8">
         <v>46073.684170520835</v>
@@ -3682,16 +3682,16 @@
         <v>46182.6840615625</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="H39" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="I39" s="8">
         <v>46002</v>
@@ -3709,13 +3709,13 @@
         <v>26</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="P39" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Q39" s="9"/>
       <c r="R39" s="9"/>
@@ -3723,15 +3723,15 @@
         <v>0</v>
       </c>
       <c r="T39" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U39" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B40" s="5">
         <v>46076.61481881945</v>
@@ -3743,16 +3743,16 @@
         <v>46127.16789894676</v>
       </c>
       <c r="E40" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G40" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="F40" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G40" s="6" t="s">
+      <c r="H40" s="6" t="s">
         <v>151</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>152</v>
       </c>
       <c r="I40" s="5">
         <v>46001</v>
@@ -3770,13 +3770,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Q40" s="5">
         <v>46001</v>
@@ -3796,7 +3796,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B41" s="8">
         <v>46076.614840277776</v>
@@ -3808,16 +3808,16 @@
         <v>46107.80900657407</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="H41" s="9" t="s">
         <v>151</v>
-      </c>
-      <c r="H41" s="9" t="s">
-        <v>152</v>
       </c>
       <c r="I41" s="8">
         <v>46001</v>
@@ -3835,13 +3835,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="Q41" s="8">
         <v>46001</v>
@@ -3853,15 +3853,15 @@
         <v>0</v>
       </c>
       <c r="T41" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U41" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B42" s="5">
         <v>46076.6150438426</v>
@@ -3873,16 +3873,16 @@
         <v>46107.80904144676</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="H42" s="6" t="s">
         <v>151</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>152</v>
       </c>
       <c r="I42" s="5">
         <v>46044</v>
@@ -3900,13 +3900,13 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="Q42" s="5">
         <v>46044</v>
@@ -3918,15 +3918,15 @@
         <v>0</v>
       </c>
       <c r="T42" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U42" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B43" s="8">
         <v>46073.68417068287</v>
@@ -3938,16 +3938,16 @@
         <v>46154.86694947917</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="H43" s="9" t="s">
         <v>151</v>
-      </c>
-      <c r="H43" s="9" t="s">
-        <v>152</v>
       </c>
       <c r="I43" s="8">
         <v>46001</v>
@@ -3965,13 +3965,13 @@
         <v>26</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="P43" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Q43" s="8">
         <v>46001</v>
@@ -3991,7 +3991,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B44" s="5">
         <v>46073.6841709375</v>
@@ -4003,16 +4003,16 @@
         <v>46107.81013429398</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="H44" s="6" t="s">
         <v>151</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>152</v>
       </c>
       <c r="I44" s="5">
         <v>46001</v>
@@ -4030,13 +4030,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4044,15 +4044,15 @@
         <v>0</v>
       </c>
       <c r="T44" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U44" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B45" s="8">
         <v>46073.68417122685</v>
@@ -4064,16 +4064,16 @@
         <v>46154.866921967594</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="H45" s="9" t="s">
         <v>151</v>
-      </c>
-      <c r="H45" s="9" t="s">
-        <v>152</v>
       </c>
       <c r="I45" s="8">
         <v>46027</v>
@@ -4091,13 +4091,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P45" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Q45" s="9"/>
       <c r="R45" s="9"/>
@@ -4105,15 +4105,15 @@
         <v>0</v>
       </c>
       <c r="T45" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U45" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B46" s="5">
         <v>46073.68417148148</v>
@@ -4125,7 +4125,7 @@
         <v>46198.57100354167</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>25</v>
@@ -4149,7 +4149,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4166,7 +4166,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B47" s="8">
         <v>46073.68417173611</v>
@@ -4178,16 +4178,16 @@
         <v>46107.72069699074</v>
       </c>
       <c r="E47" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G47" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="F47" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G47" s="9" t="s">
+      <c r="H47" s="9" t="s">
         <v>174</v>
-      </c>
-      <c r="H47" s="9" t="s">
-        <v>175</v>
       </c>
       <c r="I47" s="8">
         <v>45999</v>
@@ -4205,13 +4205,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P47" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Q47" s="8">
         <v>45999</v>
@@ -4231,7 +4231,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B48" s="5">
         <v>46073.68416831018</v>
@@ -4243,16 +4243,16 @@
         <v>46245.566249745374</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="H48" s="6" t="s">
         <v>174</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>175</v>
       </c>
       <c r="I48" s="5">
         <v>46063</v>
@@ -4270,13 +4270,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="O48" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="P48" s="6" t="s">
         <v>179</v>
-      </c>
-      <c r="P48" s="6" t="s">
-        <v>180</v>
       </c>
       <c r="Q48" s="5">
         <v>46063</v>
@@ -4296,7 +4296,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B49" s="8">
         <v>46091.74401927083</v>
@@ -4308,16 +4308,16 @@
         <v>46107.72081601852</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="H49" s="9" t="s">
         <v>174</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>175</v>
       </c>
       <c r="I49" s="9"/>
       <c r="J49" s="8">
@@ -4333,13 +4333,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="O49" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="P49" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Q49" s="8">
         <v>46070</v>
@@ -4359,7 +4359,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B50" s="5">
         <v>46091.744054490744</v>
@@ -4371,16 +4371,16 @@
         <v>46198.57098844908</v>
       </c>
       <c r="E50" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G50" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F50" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G50" s="6" t="s">
+      <c r="H50" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="I50" s="5">
         <v>46157</v>
@@ -4398,13 +4398,13 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="O50" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="P50" s="6" t="s">
         <v>188</v>
-      </c>
-      <c r="P50" s="6" t="s">
-        <v>189</v>
       </c>
       <c r="Q50" s="5">
         <v>46157</v>
@@ -4424,7 +4424,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B51" s="8">
         <v>46073.68416862268</v>
@@ -4436,7 +4436,7 @@
         <v>46127.77592181713</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>25</v>
@@ -4460,7 +4460,7 @@
         <v>26</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="P51" s="9" t="s">
         <v>26</v>
@@ -4477,7 +4477,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B52" s="5">
         <v>46073.68416885417</v>
@@ -4489,16 +4489,16 @@
         <v>46154.866942974535</v>
       </c>
       <c r="E52" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G52" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="F52" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G52" s="6" t="s">
+      <c r="H52" s="6" t="s">
         <v>195</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>196</v>
       </c>
       <c r="I52" s="5">
         <v>46057</v>
@@ -4516,13 +4516,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Q52" s="5">
         <v>46057</v>
@@ -4537,7 +4537,7 @@
         <v>32</v>
       </c>
       <c r="U52" s="12" t="s">
-        <v>59</v>
+        <v>197</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
@@ -4581,10 +4581,10 @@
         <v>26</v>
       </c>
       <c r="N53" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P53" s="9" t="s">
         <v>202</v>
@@ -4867,7 +4867,7 @@
         <v>46245.56634005787</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>25</v>
@@ -4926,10 +4926,10 @@
         <v>26</v>
       </c>
       <c r="G59" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="H59" s="9" t="s">
         <v>195</v>
-      </c>
-      <c r="H59" s="9" t="s">
-        <v>196</v>
       </c>
       <c r="I59" s="8">
         <v>46122</v>
@@ -4947,10 +4947,10 @@
         <v>26</v>
       </c>
       <c r="N59" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O59" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P59" s="9" t="s">
         <v>223</v>
@@ -4991,10 +4991,10 @@
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="H60" s="6" t="s">
         <v>195</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>196</v>
       </c>
       <c r="I60" s="5">
         <v>46058</v>
@@ -5012,10 +5012,10 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>226</v>
@@ -5056,10 +5056,10 @@
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="H61" s="9" t="s">
         <v>195</v>
-      </c>
-      <c r="H61" s="9" t="s">
-        <v>196</v>
       </c>
       <c r="I61" s="8">
         <v>46150</v>
@@ -5077,10 +5077,10 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P61" s="9" t="s">
         <v>229</v>
@@ -5121,10 +5121,10 @@
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>195</v>
-      </c>
-      <c r="H62" s="6" t="s">
-        <v>196</v>
       </c>
       <c r="I62" s="5">
         <v>46100</v>
@@ -5142,10 +5142,10 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>231</v>
@@ -5186,10 +5186,10 @@
         <v>26</v>
       </c>
       <c r="G63" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="H63" s="9" t="s">
         <v>195</v>
-      </c>
-      <c r="H63" s="9" t="s">
-        <v>196</v>
       </c>
       <c r="I63" s="8">
         <v>46126</v>
@@ -5207,10 +5207,10 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P63" s="9" t="s">
         <v>234</v>
@@ -5304,10 +5304,10 @@
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="H65" s="9" t="s">
         <v>92</v>
-      </c>
-      <c r="H65" s="9" t="s">
-        <v>93</v>
       </c>
       <c r="I65" s="8">
         <v>46094</v>
@@ -5369,10 +5369,10 @@
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H66" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="I66" s="5">
         <v>46154</v>
@@ -5434,10 +5434,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="H67" s="9" t="s">
         <v>92</v>
-      </c>
-      <c r="H67" s="9" t="s">
-        <v>93</v>
       </c>
       <c r="I67" s="8">
         <v>46126</v>
@@ -5499,10 +5499,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="I68" s="5">
         <v>46133</v>
@@ -5564,10 +5564,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="H69" s="9" t="s">
         <v>92</v>
-      </c>
-      <c r="H69" s="9" t="s">
-        <v>93</v>
       </c>
       <c r="I69" s="8">
         <v>46129</v>
@@ -5623,16 +5623,16 @@
         <v>46237.53381008102</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H70" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="I70" s="5">
         <v>46156</v>
@@ -5688,16 +5688,16 @@
         <v>46237.53382534722</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="H71" s="9" t="s">
         <v>92</v>
-      </c>
-      <c r="H71" s="9" t="s">
-        <v>93</v>
       </c>
       <c r="I71" s="8">
         <v>46160</v>
@@ -5718,7 +5718,7 @@
         <v>236</v>
       </c>
       <c r="O71" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="P71" s="9" t="s">
         <v>258</v>
@@ -5828,7 +5828,7 @@
         <v>260</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="P73" s="9" t="s">
         <v>266</v>
@@ -5867,10 +5867,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="I74" s="6"/>
       <c r="J74" s="5">
@@ -5907,7 +5907,7 @@
         <v>32</v>
       </c>
       <c r="U74" s="12" t="s">
-        <v>59</v>
+        <v>197</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -6033,7 +6033,7 @@
         <v>32</v>
       </c>
       <c r="U76" s="12" t="s">
-        <v>59</v>
+        <v>197</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -6143,7 +6143,7 @@
         <v>32</v>
       </c>
       <c r="U78" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6206,7 +6206,7 @@
         <v>32</v>
       </c>
       <c r="U79" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>